<commit_message>
M7 step 2: ERP B fields mapped (ISO country codes, VAT cleanup, payment terms keys, commodity to material group)
</commit_message>
<xml_diff>
--- a/excel/SAP_S4HANA_Mapping.xlsx
+++ b/excel/SAP_S4HANA_Mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73771AD0-F876-C240-AF39-04AF09BEAF8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{625978BE-04A7-A444-90BD-EC5D0B78461A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="261" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="172">
   <si>
     <t>Source system</t>
   </si>
@@ -469,9 +469,6 @@
     <t>LFA1-LIFNR</t>
   </si>
   <si>
-    <t>FLVN01</t>
-  </si>
-  <si>
     <t>New BP number; keep old number as reference</t>
   </si>
   <si>
@@ -518,6 +515,30 @@
   </si>
   <si>
     <t>General data (all roles)</t>
+  </si>
+  <si>
+    <t>Map country names to ISO codes (e.g. Germany → DE)</t>
+  </si>
+  <si>
+    <t>If empty: request value from supplier; if wrong length: correct postcode</t>
+  </si>
+  <si>
+    <t>Remove spaces; if empty: request value from supplier / purchasing</t>
+  </si>
+  <si>
+    <t>Map text to SAP payment terms key (e.g. "2% 14 days, net 30" → SK14)</t>
+  </si>
+  <si>
+    <t>Purchasing data (material group)</t>
+  </si>
+  <si>
+    <t>EKPO-MATKL</t>
+  </si>
+  <si>
+    <t>Not BP data</t>
+  </si>
+  <si>
+    <t>Map commodity text to a material group key</t>
   </si>
 </sst>
 </file>
@@ -944,9 +965,10 @@
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="26" customWidth="1"/>
-    <col min="4" max="5" width="22" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="25.5" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="12" customWidth="1"/>
+    <col min="7" max="7" width="21.33203125" customWidth="1"/>
     <col min="8" max="8" width="76.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -996,10 +1018,10 @@
         <v>147</v>
       </c>
       <c r="G2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
@@ -1019,13 +1041,13 @@
         <v>146</v>
       </c>
       <c r="F3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
@@ -1045,13 +1067,13 @@
         <v>146</v>
       </c>
       <c r="F4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.2">
@@ -1071,13 +1093,13 @@
         <v>146</v>
       </c>
       <c r="F5" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -1097,13 +1119,13 @@
         <v>146</v>
       </c>
       <c r="F6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -1123,13 +1145,13 @@
         <v>146</v>
       </c>
       <c r="F7" t="s">
+        <v>154</v>
+      </c>
+      <c r="G7" t="s">
+        <v>163</v>
+      </c>
+      <c r="H7" t="s">
         <v>155</v>
-      </c>
-      <c r="G7" t="s">
-        <v>164</v>
-      </c>
-      <c r="H7" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
@@ -1149,13 +1171,13 @@
         <v>146</v>
       </c>
       <c r="F8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.2">
@@ -1175,13 +1197,13 @@
         <v>146</v>
       </c>
       <c r="F9" t="s">
+        <v>157</v>
+      </c>
+      <c r="G9" t="s">
         <v>158</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>159</v>
-      </c>
-      <c r="H9" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
@@ -1198,13 +1220,13 @@
         <v>146</v>
       </c>
       <c r="F10" t="s">
+        <v>161</v>
+      </c>
+      <c r="G10" t="s">
+        <v>163</v>
+      </c>
+      <c r="H10" t="s">
         <v>162</v>
-      </c>
-      <c r="G10" t="s">
-        <v>164</v>
-      </c>
-      <c r="H10" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.2">
@@ -1223,8 +1245,13 @@
       <c r="E11" t="s">
         <v>146</v>
       </c>
-      <c r="F11" s="2"/>
+      <c r="F11" t="s">
+        <v>147</v>
+      </c>
       <c r="G11" t="s">
+        <v>163</v>
+      </c>
+      <c r="H11" t="s">
         <v>148</v>
       </c>
     </row>
@@ -1244,9 +1271,14 @@
       <c r="E12" t="s">
         <v>146</v>
       </c>
-      <c r="F12" s="2"/>
+      <c r="F12" t="s">
+        <v>150</v>
+      </c>
       <c r="G12" t="s">
-        <v>148</v>
+        <v>163</v>
+      </c>
+      <c r="H12" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
@@ -1265,9 +1297,14 @@
       <c r="E13" t="s">
         <v>146</v>
       </c>
-      <c r="F13" s="2"/>
+      <c r="F13" t="s">
+        <v>151</v>
+      </c>
       <c r="G13" t="s">
-        <v>148</v>
+        <v>163</v>
+      </c>
+      <c r="H13" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
@@ -1286,9 +1323,14 @@
       <c r="E14" t="s">
         <v>146</v>
       </c>
-      <c r="F14" s="2"/>
+      <c r="F14" t="s">
+        <v>152</v>
+      </c>
       <c r="G14" t="s">
-        <v>148</v>
+        <v>163</v>
+      </c>
+      <c r="H14" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
@@ -1307,9 +1349,14 @@
       <c r="E15" t="s">
         <v>146</v>
       </c>
-      <c r="F15" s="2"/>
+      <c r="F15" t="s">
+        <v>153</v>
+      </c>
       <c r="G15" t="s">
-        <v>148</v>
+        <v>163</v>
+      </c>
+      <c r="H15" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.2">
@@ -1325,11 +1372,20 @@
       <c r="D16" t="s">
         <v>26</v>
       </c>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E16" t="s">
+        <v>146</v>
+      </c>
+      <c r="F16" t="s">
+        <v>154</v>
+      </c>
+      <c r="G16" t="s">
+        <v>163</v>
+      </c>
+      <c r="H16" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>35</v>
       </c>
@@ -1342,11 +1398,20 @@
       <c r="D17" t="s">
         <v>29</v>
       </c>
-      <c r="E17" s="2"/>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E17" t="s">
+        <v>146</v>
+      </c>
+      <c r="F17" t="s">
+        <v>156</v>
+      </c>
+      <c r="G17" t="s">
+        <v>163</v>
+      </c>
+      <c r="H17" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>35</v>
       </c>
@@ -1359,11 +1424,20 @@
       <c r="D18" t="s">
         <v>32</v>
       </c>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E18" t="s">
+        <v>146</v>
+      </c>
+      <c r="F18" t="s">
+        <v>157</v>
+      </c>
+      <c r="G18" t="s">
+        <v>158</v>
+      </c>
+      <c r="H18" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>35</v>
       </c>
@@ -1373,9 +1447,18 @@
       <c r="C19" t="s">
         <v>51</v>
       </c>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
+      <c r="E19" t="s">
+        <v>168</v>
+      </c>
+      <c r="F19" t="s">
+        <v>169</v>
+      </c>
+      <c r="G19" t="s">
+        <v>170</v>
+      </c>
+      <c r="H19" t="s">
+        <v>171</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
M7 step 3: project steps mapped to S/4HANA apps and transactions (MDG, Migration Cockpit, ME21N, MIGO, QM notifications); README updated
</commit_message>
<xml_diff>
--- a/excel/SAP_S4HANA_Mapping.xlsx
+++ b/excel/SAP_S4HANA_Mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac1/Desktop/app_projects/supplier-data-health-check/excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{625978BE-04A7-A444-90BD-EC5D0B78461A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ED90B25-3D17-8944-BA02-6CB717D73CB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16140" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Field_Mapping" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="196">
   <si>
     <t>Source system</t>
   </si>
@@ -539,6 +539,78 @@
   </si>
   <si>
     <t>Map commodity text to a material group key</t>
+  </si>
+  <si>
+    <t>SAP MDG (data quality rules, duplicate check)</t>
+  </si>
+  <si>
+    <t>Business Partner</t>
+  </si>
+  <si>
+    <t>In the project: Python rules (M1) before migration</t>
+  </si>
+  <si>
+    <t>Migration Cockpit ("Migrate Your Data" app)</t>
+  </si>
+  <si>
+    <t>Migration object "Supplier"</t>
+  </si>
+  <si>
+    <t>Load the 120 golden records and check errors before posting</t>
+  </si>
+  <si>
+    <t>ME21N / ME23N (create / display purchase order)</t>
+  </si>
+  <si>
+    <t>EKKO, EKPO, EKET-EINDT</t>
+  </si>
+  <si>
+    <t>promised_date = planned delivery date</t>
+  </si>
+  <si>
+    <t>MIGO (goods receipt, movement type 101)</t>
+  </si>
+  <si>
+    <t>MATDOC (material document)</t>
+  </si>
+  <si>
+    <t>delivery_date and qty_received</t>
+  </si>
+  <si>
+    <t>MIGO return delivery (movement type 122) or QM inspection lot</t>
+  </si>
+  <si>
+    <t>MATDOC / QALS</t>
+  </si>
+  <si>
+    <t>PPM = rejected / received x 1,000,000</t>
+  </si>
+  <si>
+    <t>Supplier evaluation (Fiori apps)</t>
+  </si>
+  <si>
+    <t>Supplier evaluation scores</t>
+  </si>
+  <si>
+    <t>Compare with M2: delivery time and quality</t>
+  </si>
+  <si>
+    <t>QM01 / QM02 / QM03</t>
+  </si>
+  <si>
+    <t>QMEL, notification type Q2</t>
+  </si>
+  <si>
+    <t>AI (M3) could suggest the category; a person confirms</t>
+  </si>
+  <si>
+    <t>No standard S/4HANA tool: MDG change request or a ticket tool</t>
+  </si>
+  <si>
+    <t>n/a</t>
+  </si>
+  <si>
+    <t>In the project: Excel tracker (M4)</t>
   </si>
 </sst>
 </file>
@@ -561,7 +633,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -571,11 +643,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -591,12 +658,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1474,10 +1540,10 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="60" customWidth="1"/>
-    <col min="3" max="3" width="30" customWidth="1"/>
-    <col min="4" max="4" width="22" customWidth="1"/>
-    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="2" max="2" width="65.1640625" customWidth="1"/>
+    <col min="3" max="3" width="49.6640625" customWidth="1"/>
+    <col min="4" max="4" width="31.83203125" customWidth="1"/>
+    <col min="5" max="5" width="48.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="16" x14ac:dyDescent="0.2">
@@ -1504,9 +1570,15 @@
       <c r="B2" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
+      <c r="C2" t="s">
+        <v>172</v>
+      </c>
+      <c r="D2" t="s">
+        <v>173</v>
+      </c>
+      <c r="E2" t="s">
+        <v>174</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -1515,9 +1587,15 @@
       <c r="B3" t="s">
         <v>59</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
+      <c r="C3" t="s">
+        <v>175</v>
+      </c>
+      <c r="D3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E3" t="s">
+        <v>177</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -1526,9 +1604,15 @@
       <c r="B4" t="s">
         <v>61</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
+      <c r="C4" t="s">
+        <v>178</v>
+      </c>
+      <c r="D4" t="s">
+        <v>179</v>
+      </c>
+      <c r="E4" t="s">
+        <v>180</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -1537,9 +1621,15 @@
       <c r="B5" t="s">
         <v>62</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
+      <c r="C5" t="s">
+        <v>181</v>
+      </c>
+      <c r="D5" t="s">
+        <v>182</v>
+      </c>
+      <c r="E5" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
@@ -1548,9 +1638,15 @@
       <c r="B6" t="s">
         <v>63</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
+      <c r="C6" t="s">
+        <v>184</v>
+      </c>
+      <c r="D6" t="s">
+        <v>185</v>
+      </c>
+      <c r="E6" t="s">
+        <v>186</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -1559,9 +1655,15 @@
       <c r="B7" t="s">
         <v>64</v>
       </c>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
+      <c r="C7" t="s">
+        <v>187</v>
+      </c>
+      <c r="D7" t="s">
+        <v>188</v>
+      </c>
+      <c r="E7" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -1570,9 +1672,15 @@
       <c r="B8" t="s">
         <v>66</v>
       </c>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
+      <c r="C8" t="s">
+        <v>190</v>
+      </c>
+      <c r="D8" t="s">
+        <v>191</v>
+      </c>
+      <c r="E8" t="s">
+        <v>192</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -1581,9 +1689,15 @@
       <c r="B9" t="s">
         <v>68</v>
       </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
+      <c r="C9" t="s">
+        <v>193</v>
+      </c>
+      <c r="D9" t="s">
+        <v>194</v>
+      </c>
+      <c r="E9" t="s">
+        <v>195</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1906,178 +2020,178 @@
       </c>
     </row>
     <row r="2" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="2" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="2" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="11" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A11" s="3" t="s">
+      <c r="A11" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="2" t="s">
         <v>127</v>
       </c>
     </row>
     <row r="12" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="2" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="2" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="14" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B14" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="2" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="15" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A15" s="3" t="s">
+      <c r="A15" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="2" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="16" spans="1:3" ht="32" x14ac:dyDescent="0.2">
-      <c r="A16" s="3" t="s">
+      <c r="A16" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B16" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="2" t="s">
         <v>142</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A17" s="3" t="s">
+      <c r="A17" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="2" t="s">
         <v>145</v>
       </c>
     </row>

</xml_diff>